<commit_message>
Update: Added Excel Data Reader
</commit_message>
<xml_diff>
--- a/src/test/resources/UrbanLadder_TestData.xlsx
+++ b/src/test/resources/UrbanLadder_TestData.xlsx
@@ -5,15 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497838\eclipse-workspace\Display-Bookshelves\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497737\IdeaProjects\Display-Bookshelves\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3086E4F-67AD-494B-8B50-1A425B4B7D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MenuData" sheetId="1" r:id="rId1"/>
+    <sheet name="Cities" sheetId="2" r:id="rId2"/>
+    <sheet name="Bookshelves" sheetId="3" r:id="rId3"/>
+    <sheet name="StudyChairs" sheetId="4" r:id="rId4"/>
+    <sheet name="GiftCard" sheetId="5" r:id="rId5"/>
+    <sheet name="SenderReceiver" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="67">
   <si>
     <t>Expected_Oasis_Items</t>
   </si>
@@ -43,6 +48,189 @@
   </si>
   <si>
     <t>Dining Room</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Alibaug</t>
+  </si>
+  <si>
+    <t>Ambarnath</t>
+  </si>
+  <si>
+    <t>Arnala</t>
+  </si>
+  <si>
+    <t>Aurangabad</t>
+  </si>
+  <si>
+    <t>Badlapur</t>
+  </si>
+  <si>
+    <t>Boisar</t>
+  </si>
+  <si>
+    <t>Kalyan</t>
+  </si>
+  <si>
+    <t>Kamshet</t>
+  </si>
+  <si>
+    <t>Karad</t>
+  </si>
+  <si>
+    <t>Karjat</t>
+  </si>
+  <si>
+    <t>Khopoli</t>
+  </si>
+  <si>
+    <t>Koyal</t>
+  </si>
+  <si>
+    <t>Lavasa</t>
+  </si>
+  <si>
+    <t>Lonavla</t>
+  </si>
+  <si>
+    <t>Malegaon</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Nagpur</t>
+  </si>
+  <si>
+    <t>Nashik</t>
+  </si>
+  <si>
+    <t>Palghar</t>
+  </si>
+  <si>
+    <t>Pen</t>
+  </si>
+  <si>
+    <t>Pune</t>
+  </si>
+  <si>
+    <t>Raigad</t>
+  </si>
+  <si>
+    <t>Ratnagiri</t>
+  </si>
+  <si>
+    <t>Sangli</t>
+  </si>
+  <si>
+    <t>Sindhudurg</t>
+  </si>
+  <si>
+    <t>Thane</t>
+  </si>
+  <si>
+    <t>Uran</t>
+  </si>
+  <si>
+    <t>Vasai</t>
+  </si>
+  <si>
+    <t>Virar</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>MinPrice</t>
+  </si>
+  <si>
+    <t>MaxPrice</t>
+  </si>
+  <si>
+    <t>SearchText</t>
+  </si>
+  <si>
+    <t>Bookshelves</t>
+  </si>
+  <si>
+    <t>Study Chair</t>
+  </si>
+  <si>
+    <t>Denomination</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>DeliveryOption</t>
+  </si>
+  <si>
+    <t>DeliveryMode</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>gift</t>
+  </si>
+  <si>
+    <t>both</t>
+  </si>
+  <si>
+    <t>birthday</t>
+  </si>
+  <si>
+    <t>SenderFirstName</t>
+  </si>
+  <si>
+    <t>SenderLastName</t>
+  </si>
+  <si>
+    <t>SenderEmail</t>
+  </si>
+  <si>
+    <t>SenderMobile</t>
+  </si>
+  <si>
+    <t>ReceiverFirstName</t>
+  </si>
+  <si>
+    <t>ReceiverLastName</t>
+  </si>
+  <si>
+    <t>ReceiverEmail</t>
+  </si>
+  <si>
+    <t>ReceiverMobile</t>
+  </si>
+  <si>
+    <t>Message</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Wick</t>
+  </si>
+  <si>
+    <t>johnwick@abc.com</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Sparrow</t>
+  </si>
+  <si>
+    <t>jacksparrow@abc.com</t>
+  </si>
+  <si>
+    <t>Happy Birthday</t>
   </si>
 </sst>
 </file>
@@ -84,9 +272,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -406,4 +597,480 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53383EC4-5098-431A-9774-010954005067}">
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="35.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4FC8CC-9F51-457B-8F16-F0D69CBA5DFD}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.36328125" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2">
+        <v>15000</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A252B8FC-7F82-44EC-B821-FE8977DDCFDD}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.6328125" customWidth="1"/>
+    <col min="2" max="2" width="20.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="2">
+        <v>15000</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494CB382-9A20-4489-91CE-88DF03BDE76D}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.54296875" customWidth="1"/>
+    <col min="2" max="2" width="20.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BAFC188-A3E6-4034-A354-F4BEC126265B}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="35.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="2">
+        <v>8903552329</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="2">
+        <v>8903552328</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update: Implemented Data Reading From Excel
</commit_message>
<xml_diff>
--- a/src/test/resources/UrbanLadder_TestData.xlsx
+++ b/src/test/resources/UrbanLadder_TestData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497737\IdeaProjects\Display-Bookshelves\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497751_cognizant_com/Documents/Documents/Eclipse/Display-Bookshelves/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D108050-7B1E-46F9-B649-11476382470D}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MenuData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t>Expected_Oasis_Items</t>
   </si>
@@ -231,16 +231,36 @@
   </si>
   <si>
     <t>Happy Birthday</t>
+  </si>
+  <si>
+    <t>InvalidEmail</t>
+  </si>
+  <si>
+    <t>john@abccom</t>
+  </si>
+  <si>
+    <t>ExpectedErrorMessage</t>
+  </si>
+  <si>
+    <t>Enter valid Email ID.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -269,17 +289,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -559,37 +584,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -602,157 +627,157 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53383EC4-5098-431A-9774-010954005067}">
   <dimension ref="A1:A30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -765,13 +790,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4FC8CC-9F51-457B-8F16-F0D69CBA5DFD}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.36328125" customWidth="1"/>
-    <col min="2" max="2" width="16.08984375" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -780,7 +805,7 @@
       </c>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
@@ -789,7 +814,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>39</v>
       </c>
@@ -798,7 +823,7 @@
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>40</v>
       </c>
@@ -807,12 +832,12 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -825,13 +850,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A252B8FC-7F82-44EC-B821-FE8977DDCFDD}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.6328125" customWidth="1"/>
-    <col min="2" max="2" width="20.90625" customWidth="1"/>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -840,7 +865,7 @@
       </c>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
@@ -849,7 +874,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>39</v>
       </c>
@@ -858,7 +883,7 @@
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>40</v>
       </c>
@@ -867,7 +892,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -880,13 +905,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494CB382-9A20-4489-91CE-88DF03BDE76D}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.7265625" customWidth="1"/>
+    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -896,7 +921,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>
@@ -906,7 +931,7 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>44</v>
       </c>
@@ -916,7 +941,7 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>45</v>
       </c>
@@ -926,7 +951,7 @@
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>46</v>
       </c>
@@ -936,7 +961,7 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>47</v>
       </c>
@@ -946,19 +971,19 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -972,13 +997,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BAFC188-A3E6-4034-A354-F4BEC126265B}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="35.81640625" customWidth="1"/>
+    <col min="2" max="2" width="35.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
@@ -986,7 +1011,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>51</v>
       </c>
@@ -994,7 +1019,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>52</v>
       </c>
@@ -1002,7 +1027,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>53</v>
       </c>
@@ -1010,7 +1035,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>54</v>
       </c>
@@ -1018,7 +1043,7 @@
         <v>8903552329</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
@@ -1026,7 +1051,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>56</v>
       </c>
@@ -1034,7 +1059,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>57</v>
       </c>
@@ -1042,7 +1067,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>58</v>
       </c>
@@ -1050,7 +1075,7 @@
         <v>8903552328</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>59</v>
       </c>
@@ -1058,19 +1083,30 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B11" r:id="rId1" xr:uid="{AA101F7E-2577-4ACC-B691-56FC125D4CC8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update: Updated with selecting date function
</commit_message>
<xml_diff>
--- a/src/test/resources/UrbanLadder_TestData.xlsx
+++ b/src/test/resources/UrbanLadder_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497751_cognizant_com/Documents/Documents/Eclipse/Display-Bookshelves/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D108050-7B1E-46F9-B649-11476382470D}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EBFC41C-18D5-4890-AACA-188B99DFAAF7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="27165" yWindow="4800" windowWidth="17280" windowHeight="10500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MenuData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="73">
   <si>
     <t>Expected_Oasis_Items</t>
   </si>
@@ -243,6 +243,12 @@
   </si>
   <si>
     <t>Enter valid Email ID.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>19/07/2026</t>
   </si>
 </sst>
 </file>
@@ -293,13 +299,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -972,8 +981,12 @@
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>72</v>
+      </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update: Removed hardcoded values and Updated to Excel inputs
</commit_message>
<xml_diff>
--- a/src/test/resources/UrbanLadder_TestData.xlsx
+++ b/src/test/resources/UrbanLadder_TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/2497751_cognizant_com/Documents/Documents/Eclipse/Display-Bookshelves/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EBFC41C-18D5-4890-AACA-188B99DFAAF7}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="13_ncr:1_{F89414B0-CD50-419E-857A-76C060F30BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6700DC99-F99D-4BF7-9740-ABF60C62D941}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="27165" yWindow="4800" windowWidth="17280" windowHeight="10500" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MenuData" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="75">
   <si>
     <t>Expected_Oasis_Items</t>
   </si>
@@ -249,6 +249,12 @@
   </si>
   <si>
     <t>19/07/2026</t>
+  </si>
+  <si>
+    <t>ExpectedEmail</t>
+  </si>
+  <si>
+    <t>bulk@urbanladder.com</t>
   </si>
 </sst>
 </file>
@@ -299,7 +305,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -309,6 +315,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -802,7 +811,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" customWidth="1"/>
+    <col min="2" max="2" width="20.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -842,8 +851,12 @@
       <c r="C4" s="2"/>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>74</v>
+      </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -852,6 +865,9 @@
       <c r="C6" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{1161D520-CDC5-498A-B87D-9BEBD7A15E6D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>